<commit_message>
docs(evaluacion): la hoja nombra a los revisores como agente A y agente B
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/evaluacion/revision-afirmaciones-2026-10-08.xlsx
+++ b/docs/evaluacion/revision-afirmaciones-2026-10-08.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -478,14 +478,14 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>QUIÉN REVISÓ: agentes, no una persona. Codex (gpt-6-astra) y Cursor (Grok 4.7) juzgaron por separado cada frase contra el material que vio el sistema y contra la nota original descargada el 8-oct; Claude consolidó y buscó segundas fuentes. Mientras una persona no la confirme, es una evaluación exploratoria por agentes.</t>
+          <t>QUIÉN REVISÓ: agentes, no una persona. Dos agentes de IA juzgaron por separado cada frase contra el material que vio el sistema y contra la nota original descargada el 8-oct; luego se consolidó con segundas fuentes. Mientras una persona no la confirme, es una evaluación exploratoria por agentes.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Cuentan 24: A01–A23 y R1 (A24 duplica la afirmación de Mulino/Vietnam de Jeff). Con las 6 de Jeff suman 30.</t>
+          <t>El resultado es solo de 24 afirmaciones: A01–A23 y R1 (A24 quedó fuera porque repite la de Mulino y Vietnam).</t>
         </is>
       </c>
     </row>
@@ -506,7 +506,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Concordancia entre Codex y Cursor en el veredicto: 21 de 25. Diferencias: A01 (Codex: Respaldo parcial; Cursor: No respaldada), A11 (Codex: Respaldada por el material citado; Cursor: Respaldo parcial), A16 (Codex: Respaldo parcial; Cursor: Respaldada por el material citado), A17 (Codex: Respaldada por el material citado; Cursor: Respaldo parcial).</t>
+          <t>Concordancia entre los dos agentes en el veredicto: 21 de 25 filas (incluida A24). Diferencias: A01 (A: Respaldo parcial; B: No respaldada), A11 (A: Respaldada por el material citado; B: Respaldo parcial), A16 (A: Respaldo parcial; B: Respaldada por el material citado), A17 (A: Respaldada por el material citado; B: Respaldo parcial).</t>
         </is>
       </c>
     </row>
@@ -520,14 +520,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Ninguna afirmación inventó un dato: todas salen del material citado. Los problemas están en el tiempo verbal, en la atribución del contenido pagado y en errores que ya traía la fuente.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Archivos: encargos/2026-10-08-revision-afirmaciones.{prompt,codex.out,cursor.out}.md (texto de las fuentes y respuestas literales).</t>
+          <t>En esta muestra ninguna quedó como no respaldada: los problemas están en el tiempo verbal, en la atribución del contenido pagado y en errores que ya traía la fuente.</t>
         </is>
       </c>
     </row>
@@ -776,27 +769,27 @@
       </c>
       <c r="W1" s="6" t="inlineStr">
         <is>
-          <t>veredicto_codex</t>
+          <t>veredicto_agente_A</t>
         </is>
       </c>
       <c r="X1" s="6" t="inlineStr">
         <is>
-          <t>veredicto_cursor</t>
+          <t>veredicto_agente_B</t>
         </is>
       </c>
       <c r="Y1" s="6" t="inlineStr">
         <is>
-          <t>hecho_codex</t>
+          <t>hecho_agente_A</t>
         </is>
       </c>
       <c r="Z1" s="6" t="inlineStr">
         <is>
-          <t>hecho_cursor</t>
+          <t>hecho_agente_B</t>
         </is>
       </c>
       <c r="AA1" s="6" t="inlineStr">
         <is>
-          <t>cuenta_para_las_30</t>
+          <t>cuenta_para_las_24</t>
         </is>
       </c>
     </row>
@@ -894,7 +887,7 @@
       </c>
       <c r="T2" s="7" t="inlineStr">
         <is>
-          <t>Agentes, no persona: Codex (gpt-6-astra) y Cursor (Grok 4.7) por separado + consolidación de Claude con segundas fuentes</t>
+          <t>Agentes, no persona: dos agentes de IA por separado + consolidación con segundas fuentes</t>
         </is>
       </c>
       <c r="U2" s="7" t="inlineStr">
@@ -1027,7 +1020,7 @@
       </c>
       <c r="T3" s="7" t="inlineStr">
         <is>
-          <t>Agentes, no persona: Codex (gpt-6-astra) y Cursor (Grok 4.7) por separado + consolidación de Claude con segundas fuentes</t>
+          <t>Agentes, no persona: dos agentes de IA por separado + consolidación con segundas fuentes</t>
         </is>
       </c>
       <c r="U3" s="7" t="inlineStr">
@@ -1164,7 +1157,7 @@
       </c>
       <c r="T4" s="5" t="inlineStr">
         <is>
-          <t>Agentes, no persona: Codex (gpt-6-astra) y Cursor (Grok 4.7) por separado + consolidación de Claude con segundas fuentes</t>
+          <t>Agentes, no persona: dos agentes de IA por separado + consolidación con segundas fuentes</t>
         </is>
       </c>
       <c r="U4" s="5" t="inlineStr">
@@ -1297,7 +1290,7 @@
       </c>
       <c r="T5" s="5" t="inlineStr">
         <is>
-          <t>Agentes, no persona: Codex (gpt-6-astra) y Cursor (Grok 4.7) por separado + consolidación de Claude con segundas fuentes</t>
+          <t>Agentes, no persona: dos agentes de IA por separado + consolidación con segundas fuentes</t>
         </is>
       </c>
       <c r="U5" s="5" t="inlineStr">
@@ -1434,7 +1427,7 @@
       </c>
       <c r="T6" s="5" t="inlineStr">
         <is>
-          <t>Agentes, no persona: Codex (gpt-6-astra) y Cursor (Grok 4.7) por separado + consolidación de Claude con segundas fuentes</t>
+          <t>Agentes, no persona: dos agentes de IA por separado + consolidación con segundas fuentes</t>
         </is>
       </c>
       <c r="U6" s="5" t="inlineStr">
@@ -1565,7 +1558,7 @@
       </c>
       <c r="T7" s="5" t="inlineStr">
         <is>
-          <t>Agentes, no persona: Codex (gpt-6-astra) y Cursor (Grok 4.7) por separado + consolidación de Claude con segundas fuentes</t>
+          <t>Agentes, no persona: dos agentes de IA por separado + consolidación con segundas fuentes</t>
         </is>
       </c>
       <c r="U7" s="5" t="inlineStr">
@@ -1696,7 +1689,7 @@
       </c>
       <c r="T8" s="5" t="inlineStr">
         <is>
-          <t>Agentes, no persona: Codex (gpt-6-astra) y Cursor (Grok 4.7) por separado + consolidación de Claude con segundas fuentes</t>
+          <t>Agentes, no persona: dos agentes de IA por separado + consolidación con segundas fuentes</t>
         </is>
       </c>
       <c r="U8" s="5" t="inlineStr">
@@ -1831,7 +1824,7 @@
       </c>
       <c r="T9" s="7" t="inlineStr">
         <is>
-          <t>Agentes, no persona: Codex (gpt-6-astra) y Cursor (Grok 4.7) por separado + consolidación de Claude con segundas fuentes</t>
+          <t>Agentes, no persona: dos agentes de IA por separado + consolidación con segundas fuentes</t>
         </is>
       </c>
       <c r="U9" s="7" t="inlineStr">
@@ -1962,7 +1955,7 @@
       </c>
       <c r="T10" s="5" t="inlineStr">
         <is>
-          <t>Agentes, no persona: Codex (gpt-6-astra) y Cursor (Grok 4.7) por separado + consolidación de Claude con segundas fuentes</t>
+          <t>Agentes, no persona: dos agentes de IA por separado + consolidación con segundas fuentes</t>
         </is>
       </c>
       <c r="U10" s="5" t="inlineStr">
@@ -2095,7 +2088,7 @@
       </c>
       <c r="T11" s="5" t="inlineStr">
         <is>
-          <t>Agentes, no persona: Codex (gpt-6-astra) y Cursor (Grok 4.7) por separado + consolidación de Claude con segundas fuentes</t>
+          <t>Agentes, no persona: dos agentes de IA por separado + consolidación con segundas fuentes</t>
         </is>
       </c>
       <c r="U11" s="5" t="inlineStr">
@@ -2230,7 +2223,7 @@
       </c>
       <c r="T12" s="5" t="inlineStr">
         <is>
-          <t>Agentes, no persona: Codex (gpt-6-astra) y Cursor (Grok 4.7) por separado + consolidación de Claude con segundas fuentes</t>
+          <t>Agentes, no persona: dos agentes de IA por separado + consolidación con segundas fuentes</t>
         </is>
       </c>
       <c r="U12" s="5" t="inlineStr">
@@ -2367,7 +2360,7 @@
       </c>
       <c r="T13" s="5" t="inlineStr">
         <is>
-          <t>Agentes, no persona: Codex (gpt-6-astra) y Cursor (Grok 4.7) por separado + consolidación de Claude con segundas fuentes</t>
+          <t>Agentes, no persona: dos agentes de IA por separado + consolidación con segundas fuentes</t>
         </is>
       </c>
       <c r="U13" s="5" t="inlineStr">
@@ -2502,7 +2495,7 @@
       </c>
       <c r="T14" s="5" t="inlineStr">
         <is>
-          <t>Agentes, no persona: Codex (gpt-6-astra) y Cursor (Grok 4.7) por separado + consolidación de Claude con segundas fuentes</t>
+          <t>Agentes, no persona: dos agentes de IA por separado + consolidación con segundas fuentes</t>
         </is>
       </c>
       <c r="U14" s="5" t="inlineStr">
@@ -2633,7 +2626,7 @@
       </c>
       <c r="T15" s="5" t="inlineStr">
         <is>
-          <t>Agentes, no persona: Codex (gpt-6-astra) y Cursor (Grok 4.7) por separado + consolidación de Claude con segundas fuentes</t>
+          <t>Agentes, no persona: dos agentes de IA por separado + consolidación con segundas fuentes</t>
         </is>
       </c>
       <c r="U15" s="5" t="inlineStr">
@@ -2764,7 +2757,7 @@
       </c>
       <c r="T16" s="5" t="inlineStr">
         <is>
-          <t>Agentes, no persona: Codex (gpt-6-astra) y Cursor (Grok 4.7) por separado + consolidación de Claude con segundas fuentes</t>
+          <t>Agentes, no persona: dos agentes de IA por separado + consolidación con segundas fuentes</t>
         </is>
       </c>
       <c r="U16" s="5" t="inlineStr">
@@ -2895,7 +2888,7 @@
       </c>
       <c r="T17" s="7" t="inlineStr">
         <is>
-          <t>Agentes, no persona: Codex (gpt-6-astra) y Cursor (Grok 4.7) por separado + consolidación de Claude con segundas fuentes</t>
+          <t>Agentes, no persona: dos agentes de IA por separado + consolidación con segundas fuentes</t>
         </is>
       </c>
       <c r="U17" s="7" t="inlineStr">
@@ -3030,7 +3023,7 @@
       </c>
       <c r="T18" s="5" t="inlineStr">
         <is>
-          <t>Agentes, no persona: Codex (gpt-6-astra) y Cursor (Grok 4.7) por separado + consolidación de Claude con segundas fuentes</t>
+          <t>Agentes, no persona: dos agentes de IA por separado + consolidación con segundas fuentes</t>
         </is>
       </c>
       <c r="U18" s="5" t="inlineStr">
@@ -3161,7 +3154,7 @@
       </c>
       <c r="T19" s="5" t="inlineStr">
         <is>
-          <t>Agentes, no persona: Codex (gpt-6-astra) y Cursor (Grok 4.7) por separado + consolidación de Claude con segundas fuentes</t>
+          <t>Agentes, no persona: dos agentes de IA por separado + consolidación con segundas fuentes</t>
         </is>
       </c>
       <c r="U19" s="5" t="inlineStr">
@@ -3292,7 +3285,7 @@
       </c>
       <c r="T20" s="5" t="inlineStr">
         <is>
-          <t>Agentes, no persona: Codex (gpt-6-astra) y Cursor (Grok 4.7) por separado + consolidación de Claude con segundas fuentes</t>
+          <t>Agentes, no persona: dos agentes de IA por separado + consolidación con segundas fuentes</t>
         </is>
       </c>
       <c r="U20" s="5" t="inlineStr">
@@ -3423,7 +3416,7 @@
       </c>
       <c r="T21" s="5" t="inlineStr">
         <is>
-          <t>Agentes, no persona: Codex (gpt-6-astra) y Cursor (Grok 4.7) por separado + consolidación de Claude con segundas fuentes</t>
+          <t>Agentes, no persona: dos agentes de IA por separado + consolidación con segundas fuentes</t>
         </is>
       </c>
       <c r="U21" s="5" t="inlineStr">
@@ -3554,7 +3547,7 @@
       </c>
       <c r="T22" s="5" t="inlineStr">
         <is>
-          <t>Agentes, no persona: Codex (gpt-6-astra) y Cursor (Grok 4.7) por separado + consolidación de Claude con segundas fuentes</t>
+          <t>Agentes, no persona: dos agentes de IA por separado + consolidación con segundas fuentes</t>
         </is>
       </c>
       <c r="U22" s="5" t="inlineStr">
@@ -3685,7 +3678,7 @@
       </c>
       <c r="T23" s="5" t="inlineStr">
         <is>
-          <t>Agentes, no persona: Codex (gpt-6-astra) y Cursor (Grok 4.7) por separado + consolidación de Claude con segundas fuentes</t>
+          <t>Agentes, no persona: dos agentes de IA por separado + consolidación con segundas fuentes</t>
         </is>
       </c>
       <c r="U23" s="5" t="inlineStr">
@@ -3820,7 +3813,7 @@
       </c>
       <c r="T24" s="7" t="inlineStr">
         <is>
-          <t>Agentes, no persona: Codex (gpt-6-astra) y Cursor (Grok 4.7) por separado + consolidación de Claude con segundas fuentes</t>
+          <t>Agentes, no persona: dos agentes de IA por separado + consolidación con segundas fuentes</t>
         </is>
       </c>
       <c r="U24" s="7" t="inlineStr">
@@ -3957,7 +3950,7 @@
       </c>
       <c r="T25" s="5" t="inlineStr">
         <is>
-          <t>Agentes, no persona: Codex (gpt-6-astra) y Cursor (Grok 4.7) por separado + consolidación de Claude con segundas fuentes</t>
+          <t>Agentes, no persona: dos agentes de IA por separado + consolidación con segundas fuentes</t>
         </is>
       </c>
       <c r="U25" s="5" t="inlineStr">
@@ -3967,7 +3960,7 @@
       </c>
       <c r="V25" s="5" t="inlineStr">
         <is>
-          <t>sin cambios — NO CUENTA: duplica la afirmación de Mulino/Vietnam de Jeff (se usa R1)</t>
+          <t>sin cambios — NO CUENTA: repite la afirmación de Mulino y Vietnam (se usa R1)</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
@@ -3992,7 +3985,7 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>no (duplica a Jeff)</t>
+          <t>no (repite la de Mulino y Vietnam)</t>
         </is>
       </c>
     </row>
@@ -4092,7 +4085,7 @@
       </c>
       <c r="T26" s="7" t="inlineStr">
         <is>
-          <t>Agentes, no persona: Codex (gpt-6-astra) y Cursor (Grok 4.7) por separado + consolidación de Claude con segundas fuentes</t>
+          <t>Agentes, no persona: dos agentes de IA por separado + consolidación con segundas fuentes</t>
         </is>
       </c>
       <c r="U26" s="7" t="inlineStr">

</xml_diff>